<commit_message>
Aggiornato Avanzamento.xlsx da lbianco via Streamlit
</commit_message>
<xml_diff>
--- a/Avanzamento.xlsx
+++ b/Avanzamento.xlsx
@@ -12,15 +12,15 @@
     <sheet name="Foglio3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Foglio1!$A$1:$G$507</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Foglio3!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Foglio1!$A$1:$G$651</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Foglio3!$A$36:$D$36</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1518" uniqueCount="147">
   <si>
     <t>Tecnico</t>
   </si>
@@ -948,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H507"/>
+  <dimension ref="A1:H651"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
@@ -13212,7 +13212,7 @@
         <v>20</v>
       </c>
       <c r="F497" s="3">
-        <f t="shared" ref="F497:F507" si="10">D497-(D497*E497)/100</f>
+        <f t="shared" ref="F497:F506" si="10">D497-(D497*E497)/100</f>
         <v>37.364453019576082</v>
       </c>
       <c r="G497" s="1"/>
@@ -13440,8 +13440,3460 @@
       <c r="G507" s="1"/>
       <c r="H507" s="1"/>
     </row>
+    <row r="508" spans="1:8">
+      <c r="A508" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B508" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C508" s="8">
+        <v>64</v>
+      </c>
+      <c r="D508" s="11">
+        <v>55.460559782608698</v>
+      </c>
+      <c r="E508" s="12">
+        <v>20</v>
+      </c>
+      <c r="F508" s="13">
+        <f t="shared" ref="F508:F570" si="11">D508-(D508*E508)/100</f>
+        <v>44.368447826086957</v>
+      </c>
+      <c r="G508" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H508" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="509" spans="1:8">
+      <c r="A509" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B509" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C509" s="8">
+        <v>16</v>
+      </c>
+      <c r="D509" s="4">
+        <v>45.514765360169498</v>
+      </c>
+      <c r="E509" s="6">
+        <v>20</v>
+      </c>
+      <c r="F509" s="3">
+        <f t="shared" si="11"/>
+        <v>36.4118122881356</v>
+      </c>
+      <c r="G509" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H509" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="510" spans="1:8">
+      <c r="A510" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B510" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C510" s="8">
+        <v>8</v>
+      </c>
+      <c r="D510" s="4">
+        <v>31.3675568181818</v>
+      </c>
+      <c r="E510" s="6">
+        <v>20</v>
+      </c>
+      <c r="F510" s="3">
+        <f t="shared" si="11"/>
+        <v>25.094045454545441</v>
+      </c>
+      <c r="G510" s="1"/>
+      <c r="H510" s="7"/>
+    </row>
+    <row r="511" spans="1:8">
+      <c r="A511" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B511" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C511" s="8">
+        <v>71</v>
+      </c>
+      <c r="D511" s="4">
+        <v>55.188342723004702</v>
+      </c>
+      <c r="E511" s="6">
+        <v>20</v>
+      </c>
+      <c r="F511" s="3">
+        <f t="shared" si="11"/>
+        <v>44.150674178403762</v>
+      </c>
+      <c r="G511" s="1"/>
+      <c r="H511" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="512" spans="1:8">
+      <c r="A512" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B512" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C512" s="8">
+        <v>47</v>
+      </c>
+      <c r="D512" s="4">
+        <v>39.116093220339003</v>
+      </c>
+      <c r="E512" s="6">
+        <v>20</v>
+      </c>
+      <c r="F512" s="3">
+        <f t="shared" si="11"/>
+        <v>31.292874576271203</v>
+      </c>
+      <c r="G512" s="1"/>
+      <c r="H512" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="513" spans="1:8">
+      <c r="A513" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B513" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C513" s="8">
+        <v>88</v>
+      </c>
+      <c r="D513" s="4">
+        <v>24.494655963302801</v>
+      </c>
+      <c r="E513" s="6">
+        <v>20</v>
+      </c>
+      <c r="F513" s="3">
+        <f t="shared" si="11"/>
+        <v>19.595724770642242</v>
+      </c>
+      <c r="G513" s="1"/>
+      <c r="H513" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="514" spans="1:8">
+      <c r="A514" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B514" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C514" s="8">
+        <v>104</v>
+      </c>
+      <c r="D514" s="4">
+        <v>30.3595985356387</v>
+      </c>
+      <c r="E514" s="6">
+        <v>20</v>
+      </c>
+      <c r="F514" s="3">
+        <f t="shared" si="11"/>
+        <v>24.287678828510959</v>
+      </c>
+      <c r="G514" s="1"/>
+      <c r="H514" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="515" spans="1:8">
+      <c r="A515" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B515" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C515" s="8">
+        <v>64</v>
+      </c>
+      <c r="D515" s="4">
+        <v>29.055033333333299</v>
+      </c>
+      <c r="E515" s="6">
+        <v>20</v>
+      </c>
+      <c r="F515" s="3">
+        <f t="shared" si="11"/>
+        <v>23.244026666666638</v>
+      </c>
+      <c r="G515" s="1"/>
+      <c r="H515" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="516" spans="1:8">
+      <c r="A516" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B516" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C516" s="8">
+        <v>168</v>
+      </c>
+      <c r="D516" s="4">
+        <v>24.878616379310301</v>
+      </c>
+      <c r="E516" s="6">
+        <v>20</v>
+      </c>
+      <c r="F516" s="3">
+        <f t="shared" si="11"/>
+        <v>19.902893103448243</v>
+      </c>
+      <c r="G516" s="1"/>
+      <c r="H516" s="7"/>
+    </row>
+    <row r="517" spans="1:8">
+      <c r="A517" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B517" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C517" s="8">
+        <v>112</v>
+      </c>
+      <c r="D517" s="4">
+        <v>30.848343750000002</v>
+      </c>
+      <c r="E517" s="6">
+        <v>20</v>
+      </c>
+      <c r="F517" s="3">
+        <f t="shared" si="11"/>
+        <v>24.678675000000002</v>
+      </c>
+      <c r="G517" s="1"/>
+      <c r="H517" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="518" spans="1:8">
+      <c r="A518" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B518" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C518" s="8">
+        <v>54</v>
+      </c>
+      <c r="D518" s="4">
+        <v>39.049898148148202</v>
+      </c>
+      <c r="E518" s="6">
+        <v>20</v>
+      </c>
+      <c r="F518" s="3">
+        <f t="shared" si="11"/>
+        <v>31.239918518518561</v>
+      </c>
+      <c r="G518" s="1"/>
+      <c r="H518" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="519" spans="1:8">
+      <c r="A519" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B519" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C519" s="8">
+        <v>46</v>
+      </c>
+      <c r="D519" s="4">
+        <v>28.0704130434783</v>
+      </c>
+      <c r="E519" s="6">
+        <v>20</v>
+      </c>
+      <c r="F519" s="3">
+        <f t="shared" si="11"/>
+        <v>22.45633043478264</v>
+      </c>
+      <c r="G519" s="1"/>
+      <c r="H519" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="520" spans="1:8">
+      <c r="A520" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B520" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C520" s="8">
+        <v>64</v>
+      </c>
+      <c r="D520" s="4">
+        <v>27.316808948863599</v>
+      </c>
+      <c r="E520" s="6">
+        <v>20</v>
+      </c>
+      <c r="F520" s="3">
+        <f t="shared" si="11"/>
+        <v>21.85344715909088</v>
+      </c>
+      <c r="G520" s="1"/>
+      <c r="H520" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="521" spans="1:8">
+      <c r="A521" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B521" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C521" s="8">
+        <v>88</v>
+      </c>
+      <c r="D521" s="4">
+        <v>24.494655963302801</v>
+      </c>
+      <c r="E521" s="6">
+        <v>20</v>
+      </c>
+      <c r="F521" s="3">
+        <f t="shared" si="11"/>
+        <v>19.595724770642242</v>
+      </c>
+      <c r="G521" s="1"/>
+      <c r="H521" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="522" spans="1:8">
+      <c r="A522" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B522" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C522" s="8">
+        <v>55</v>
+      </c>
+      <c r="D522" s="4">
+        <v>40.977525115562401</v>
+      </c>
+      <c r="E522" s="6">
+        <v>20</v>
+      </c>
+      <c r="F522" s="3">
+        <f t="shared" si="11"/>
+        <v>32.782020092449919</v>
+      </c>
+      <c r="G522" s="1"/>
+      <c r="H522" s="7"/>
+    </row>
+    <row r="523" spans="1:8">
+      <c r="A523" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B523" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C523" s="8">
+        <v>72</v>
+      </c>
+      <c r="D523" s="4">
+        <v>23.965367647058802</v>
+      </c>
+      <c r="E523" s="6">
+        <v>20</v>
+      </c>
+      <c r="F523" s="3">
+        <f t="shared" si="11"/>
+        <v>19.172294117647041</v>
+      </c>
+      <c r="G523" s="1"/>
+      <c r="H523" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="524" spans="1:8">
+      <c r="A524" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B524" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C524" s="8">
+        <v>88</v>
+      </c>
+      <c r="D524" s="4">
+        <v>26.892847222222201</v>
+      </c>
+      <c r="E524" s="6">
+        <v>20</v>
+      </c>
+      <c r="F524" s="3">
+        <f t="shared" si="11"/>
+        <v>21.51427777777776</v>
+      </c>
+      <c r="G524" s="1"/>
+      <c r="H524" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="525" spans="1:8">
+      <c r="A525" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B525" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C525" s="8">
+        <v>72</v>
+      </c>
+      <c r="D525" s="4">
+        <v>52.019903802685803</v>
+      </c>
+      <c r="E525" s="6">
+        <v>20</v>
+      </c>
+      <c r="F525" s="3">
+        <f t="shared" si="11"/>
+        <v>41.615923042148644</v>
+      </c>
+      <c r="G525" s="1"/>
+      <c r="H525" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="526" spans="1:8">
+      <c r="A526" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B526" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C526" s="8">
+        <v>96</v>
+      </c>
+      <c r="D526" s="4">
+        <v>37.910187317890497</v>
+      </c>
+      <c r="E526" s="6">
+        <v>20</v>
+      </c>
+      <c r="F526" s="3">
+        <f t="shared" si="11"/>
+        <v>30.328149854312397</v>
+      </c>
+      <c r="G526" s="1"/>
+      <c r="H526" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="527" spans="1:8">
+      <c r="A527" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B527" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C527" s="8">
+        <v>83</v>
+      </c>
+      <c r="D527" s="4">
+        <v>49.366206168522702</v>
+      </c>
+      <c r="E527" s="6">
+        <v>20</v>
+      </c>
+      <c r="F527" s="3">
+        <f t="shared" si="11"/>
+        <v>39.492964934818161</v>
+      </c>
+      <c r="G527" s="1"/>
+      <c r="H527" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="528" spans="1:8">
+      <c r="A528" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B528" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C528" s="8">
+        <v>112</v>
+      </c>
+      <c r="D528" s="4">
+        <v>40.497301136363603</v>
+      </c>
+      <c r="E528" s="6">
+        <v>20</v>
+      </c>
+      <c r="F528" s="3">
+        <f t="shared" si="11"/>
+        <v>32.397840909090881</v>
+      </c>
+      <c r="G528" s="1"/>
+      <c r="H528" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="529" spans="1:8">
+      <c r="A529" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B529" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C529" s="8">
+        <v>64</v>
+      </c>
+      <c r="D529" s="4">
+        <v>37.228785120902799</v>
+      </c>
+      <c r="E529" s="6">
+        <v>20</v>
+      </c>
+      <c r="F529" s="3">
+        <f t="shared" si="11"/>
+        <v>29.783028096722241</v>
+      </c>
+      <c r="G529" s="1"/>
+      <c r="H529" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="530" spans="1:8">
+      <c r="A530" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B530" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C530" s="8">
+        <v>76</v>
+      </c>
+      <c r="D530" s="4">
+        <v>31.200952114738399</v>
+      </c>
+      <c r="E530" s="6">
+        <v>20</v>
+      </c>
+      <c r="F530" s="3">
+        <f t="shared" si="11"/>
+        <v>24.960761691790719</v>
+      </c>
+      <c r="G530" s="1"/>
+      <c r="H530" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="531" spans="1:8">
+      <c r="A531" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B531" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C531" s="8">
+        <v>116</v>
+      </c>
+      <c r="D531" s="4">
+        <v>44.601379654048102</v>
+      </c>
+      <c r="E531" s="6">
+        <v>20</v>
+      </c>
+      <c r="F531" s="3">
+        <f t="shared" si="11"/>
+        <v>35.681103723238479</v>
+      </c>
+      <c r="G531" s="1"/>
+      <c r="H531" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="532" spans="1:8">
+      <c r="A532" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B532" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C532" s="8">
+        <v>8</v>
+      </c>
+      <c r="D532" s="4">
+        <v>102.1819375</v>
+      </c>
+      <c r="E532" s="6">
+        <v>20</v>
+      </c>
+      <c r="F532" s="3">
+        <f t="shared" si="11"/>
+        <v>81.745550000000009</v>
+      </c>
+      <c r="G532" s="1"/>
+      <c r="H532" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="533" spans="1:8">
+      <c r="A533" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B533" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C533" s="8"/>
+      <c r="D533" s="4"/>
+      <c r="E533" s="6">
+        <v>20</v>
+      </c>
+      <c r="F533" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G533" s="1"/>
+      <c r="H533" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="534" spans="1:8">
+      <c r="A534" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B534" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C534" s="8">
+        <v>79</v>
+      </c>
+      <c r="D534" s="4">
+        <v>26.734704805835701</v>
+      </c>
+      <c r="E534" s="6">
+        <v>20</v>
+      </c>
+      <c r="F534" s="3">
+        <f t="shared" si="11"/>
+        <v>21.387763844668562</v>
+      </c>
+      <c r="G534" s="1"/>
+      <c r="H534" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="535" spans="1:8">
+      <c r="A535" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B535" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C535" s="8">
+        <v>116</v>
+      </c>
+      <c r="D535" s="4">
+        <v>44.601379654048102</v>
+      </c>
+      <c r="E535" s="6">
+        <v>20</v>
+      </c>
+      <c r="F535" s="3">
+        <f t="shared" si="11"/>
+        <v>35.681103723238479</v>
+      </c>
+      <c r="G535" s="1"/>
+      <c r="H535" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="536" spans="1:8">
+      <c r="A536" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B536" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C536" s="8"/>
+      <c r="D536" s="4"/>
+      <c r="E536" s="6">
+        <v>20</v>
+      </c>
+      <c r="F536" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G536" s="1"/>
+      <c r="H536" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="537" spans="1:8">
+      <c r="A537" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B537" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C537" s="8">
+        <v>56</v>
+      </c>
+      <c r="D537" s="4">
+        <v>37.2749375</v>
+      </c>
+      <c r="E537" s="6">
+        <v>20</v>
+      </c>
+      <c r="F537" s="3">
+        <f t="shared" si="11"/>
+        <v>29.819949999999999</v>
+      </c>
+      <c r="G537" s="1"/>
+      <c r="H537" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="538" spans="1:8">
+      <c r="A538" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B538" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C538" s="8">
+        <v>80</v>
+      </c>
+      <c r="D538" s="4">
+        <v>37.246492480283898</v>
+      </c>
+      <c r="E538" s="6">
+        <v>20</v>
+      </c>
+      <c r="F538" s="3">
+        <f t="shared" si="11"/>
+        <v>29.797193984227118</v>
+      </c>
+      <c r="G538" s="1"/>
+      <c r="H538" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="539" spans="1:8">
+      <c r="A539" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B539" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C539" s="8">
+        <v>48</v>
+      </c>
+      <c r="D539" s="4">
+        <v>59.174228618113901</v>
+      </c>
+      <c r="E539" s="6">
+        <v>20</v>
+      </c>
+      <c r="F539" s="3">
+        <f t="shared" si="11"/>
+        <v>47.339382894491123</v>
+      </c>
+      <c r="G539" s="1"/>
+      <c r="H539" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="540" spans="1:8">
+      <c r="A540" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B540" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C540" s="8">
+        <v>136</v>
+      </c>
+      <c r="D540" s="4">
+        <v>28.483891129032301</v>
+      </c>
+      <c r="E540" s="6">
+        <v>20</v>
+      </c>
+      <c r="F540" s="3">
+        <f t="shared" si="11"/>
+        <v>22.787112903225839</v>
+      </c>
+      <c r="G540" s="1"/>
+      <c r="H540" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="541" spans="1:8">
+      <c r="A541" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B541" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C541" s="8">
+        <v>80</v>
+      </c>
+      <c r="D541" s="4">
+        <v>61.339145574229697</v>
+      </c>
+      <c r="E541" s="6">
+        <v>20</v>
+      </c>
+      <c r="F541" s="3">
+        <f t="shared" si="11"/>
+        <v>49.071316459383759</v>
+      </c>
+      <c r="G541" s="1"/>
+      <c r="H541" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="542" spans="1:8">
+      <c r="A542" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B542" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C542" s="8"/>
+      <c r="D542" s="4"/>
+      <c r="E542" s="6">
+        <v>20</v>
+      </c>
+      <c r="F542" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G542" s="1"/>
+      <c r="H542" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="543" spans="1:8">
+      <c r="A543" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B543" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C543" s="8">
+        <v>8</v>
+      </c>
+      <c r="D543" s="4">
+        <v>102.1819375</v>
+      </c>
+      <c r="E543" s="6">
+        <v>20</v>
+      </c>
+      <c r="F543" s="3">
+        <f t="shared" si="11"/>
+        <v>81.745550000000009</v>
+      </c>
+      <c r="G543" s="1"/>
+      <c r="H543" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="544" spans="1:8">
+      <c r="A544" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B544" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C544" s="8">
+        <v>75</v>
+      </c>
+      <c r="D544" s="4">
+        <v>28.6258956072644</v>
+      </c>
+      <c r="E544" s="6">
+        <v>20</v>
+      </c>
+      <c r="F544" s="3">
+        <f t="shared" si="11"/>
+        <v>22.900716485811522</v>
+      </c>
+      <c r="G544" s="1"/>
+      <c r="H544" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="545" spans="1:8">
+      <c r="A545" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B545" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C545" s="8">
+        <v>56</v>
+      </c>
+      <c r="D545" s="4">
+        <v>31.9272796610169</v>
+      </c>
+      <c r="E545" s="6">
+        <v>20</v>
+      </c>
+      <c r="F545" s="3">
+        <f t="shared" si="11"/>
+        <v>25.541823728813519</v>
+      </c>
+      <c r="G545" s="1"/>
+      <c r="H545" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="546" spans="1:8">
+      <c r="A546" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B546" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C546" s="8">
+        <v>88</v>
+      </c>
+      <c r="D546" s="4">
+        <v>31.922168861024002</v>
+      </c>
+      <c r="E546" s="6">
+        <v>20</v>
+      </c>
+      <c r="F546" s="3">
+        <f t="shared" si="11"/>
+        <v>25.537735088819201</v>
+      </c>
+      <c r="G546" s="1"/>
+      <c r="H546" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="547" spans="1:8">
+      <c r="A547" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B547" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C547" s="8">
+        <v>136</v>
+      </c>
+      <c r="D547" s="4">
+        <v>31.394258064516102</v>
+      </c>
+      <c r="E547" s="6">
+        <v>20</v>
+      </c>
+      <c r="F547" s="3">
+        <f t="shared" si="11"/>
+        <v>25.115406451612881</v>
+      </c>
+      <c r="G547" s="1"/>
+      <c r="H547" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="548" spans="1:8">
+      <c r="A548" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B548" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C548" s="8">
+        <v>8</v>
+      </c>
+      <c r="D548" s="4">
+        <v>102.1819375</v>
+      </c>
+      <c r="E548" s="6">
+        <v>20</v>
+      </c>
+      <c r="F548" s="3">
+        <f t="shared" si="11"/>
+        <v>81.745550000000009</v>
+      </c>
+      <c r="G548" s="1"/>
+      <c r="H548" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="549" spans="1:8">
+      <c r="A549" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B549" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C549" s="8">
+        <v>112</v>
+      </c>
+      <c r="D549" s="4">
+        <v>43.613494177018602</v>
+      </c>
+      <c r="E549" s="6">
+        <v>20</v>
+      </c>
+      <c r="F549" s="3">
+        <f t="shared" si="11"/>
+        <v>34.890795341614883</v>
+      </c>
+      <c r="G549" s="1"/>
+      <c r="H549" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="550" spans="1:8">
+      <c r="A550" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B550" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C550" s="8"/>
+      <c r="D550" s="4"/>
+      <c r="E550" s="6">
+        <v>20</v>
+      </c>
+      <c r="F550" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G550" s="1"/>
+      <c r="H550" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="551" spans="1:8">
+      <c r="A551" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B551" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C551" s="8">
+        <v>144</v>
+      </c>
+      <c r="D551" s="4">
+        <v>64.586521008403395</v>
+      </c>
+      <c r="E551" s="6">
+        <v>20</v>
+      </c>
+      <c r="F551" s="3">
+        <f t="shared" si="11"/>
+        <v>51.669216806722716</v>
+      </c>
+      <c r="G551" s="1"/>
+      <c r="H551" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="552" spans="1:8">
+      <c r="A552" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B552" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C552" s="8">
+        <v>78</v>
+      </c>
+      <c r="D552" s="4">
+        <v>62.088539905192803</v>
+      </c>
+      <c r="E552" s="6">
+        <v>20</v>
+      </c>
+      <c r="F552" s="3">
+        <f t="shared" si="11"/>
+        <v>49.670831924154243</v>
+      </c>
+      <c r="G552" s="1"/>
+      <c r="H552" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="553" spans="1:8">
+      <c r="A553" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B553" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C553" s="8">
+        <v>8</v>
+      </c>
+      <c r="D553" s="4">
+        <v>423.4525625</v>
+      </c>
+      <c r="E553" s="6">
+        <v>20</v>
+      </c>
+      <c r="F553" s="3">
+        <f t="shared" si="11"/>
+        <v>338.76204999999999</v>
+      </c>
+      <c r="G553" s="1"/>
+      <c r="H553" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="554" spans="1:8">
+      <c r="A554" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B554" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C554" s="8"/>
+      <c r="D554" s="4"/>
+      <c r="E554" s="6">
+        <v>20</v>
+      </c>
+      <c r="F554" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G554" s="1"/>
+      <c r="H554" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="555" spans="1:8">
+      <c r="A555" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B555" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C555" s="8"/>
+      <c r="D555" s="4"/>
+      <c r="E555" s="6">
+        <v>20</v>
+      </c>
+      <c r="F555" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G555" s="1"/>
+      <c r="H555" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="556" spans="1:8">
+      <c r="A556" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B556" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C556" s="8"/>
+      <c r="D556" s="4"/>
+      <c r="E556" s="6">
+        <v>20</v>
+      </c>
+      <c r="F556" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G556" s="1"/>
+      <c r="H556" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="557" spans="1:8">
+      <c r="A557" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B557" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C557" s="8">
+        <v>136</v>
+      </c>
+      <c r="D557" s="4">
+        <v>31.938663606654799</v>
+      </c>
+      <c r="E557" s="6">
+        <v>20</v>
+      </c>
+      <c r="F557" s="3">
+        <f t="shared" si="11"/>
+        <v>25.55093088532384</v>
+      </c>
+      <c r="G557" s="1"/>
+      <c r="H557" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="558" spans="1:8">
+      <c r="A558" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B558" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C558" s="8"/>
+      <c r="D558" s="4"/>
+      <c r="E558" s="6">
+        <v>20</v>
+      </c>
+      <c r="F558" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G558" s="1"/>
+      <c r="H558" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="559" spans="1:8">
+      <c r="A559" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B559" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C559" s="8">
+        <v>136</v>
+      </c>
+      <c r="D559" s="4">
+        <v>31.604892504530302</v>
+      </c>
+      <c r="E559" s="6">
+        <v>20</v>
+      </c>
+      <c r="F559" s="3">
+        <f t="shared" si="11"/>
+        <v>25.28391400362424</v>
+      </c>
+      <c r="G559" s="1"/>
+      <c r="H559" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="560" spans="1:8">
+      <c r="A560" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B560" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C560" s="8"/>
+      <c r="D560" s="4"/>
+      <c r="E560" s="6">
+        <v>20</v>
+      </c>
+      <c r="F560" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G560" s="1"/>
+      <c r="H560" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="561" spans="1:8">
+      <c r="A561" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B561" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C561" s="8">
+        <v>72</v>
+      </c>
+      <c r="D561" s="4">
+        <v>30.678258940532601</v>
+      </c>
+      <c r="E561" s="6">
+        <v>20</v>
+      </c>
+      <c r="F561" s="3">
+        <f t="shared" si="11"/>
+        <v>24.542607152426079</v>
+      </c>
+      <c r="G561" s="1"/>
+      <c r="H561" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="562" spans="1:8">
+      <c r="A562" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B562" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C562" s="8">
+        <v>84</v>
+      </c>
+      <c r="D562" s="4">
+        <v>20.590436744694799</v>
+      </c>
+      <c r="E562" s="6">
+        <v>20</v>
+      </c>
+      <c r="F562" s="3">
+        <f t="shared" si="11"/>
+        <v>16.472349395755838</v>
+      </c>
+      <c r="G562" s="1"/>
+      <c r="H562" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="563" spans="1:8">
+      <c r="A563" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B563" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C563" s="8">
+        <v>64</v>
+      </c>
+      <c r="D563" s="4">
+        <v>27.316808948863599</v>
+      </c>
+      <c r="E563" s="6">
+        <v>20</v>
+      </c>
+      <c r="F563" s="3">
+        <f t="shared" si="11"/>
+        <v>21.85344715909088</v>
+      </c>
+      <c r="G563" s="1"/>
+      <c r="H563" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="564" spans="1:8">
+      <c r="A564" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B564" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C564" s="8">
+        <v>80</v>
+      </c>
+      <c r="D564" s="4">
+        <v>71.595940596330294</v>
+      </c>
+      <c r="E564" s="6">
+        <v>20</v>
+      </c>
+      <c r="F564" s="3">
+        <f t="shared" si="11"/>
+        <v>57.276752477064235</v>
+      </c>
+      <c r="G564" s="1"/>
+      <c r="H564" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="565" spans="1:8">
+      <c r="A565" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B565" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C565" s="8">
+        <v>80</v>
+      </c>
+      <c r="D565" s="4">
+        <v>76.829416666666603</v>
+      </c>
+      <c r="E565" s="6">
+        <v>20</v>
+      </c>
+      <c r="F565" s="3">
+        <f t="shared" si="11"/>
+        <v>61.463533333333281</v>
+      </c>
+      <c r="G565" s="1"/>
+      <c r="H565" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="566" spans="1:8">
+      <c r="A566" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B566" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C566" s="8"/>
+      <c r="D566" s="4"/>
+      <c r="E566" s="6">
+        <v>20</v>
+      </c>
+      <c r="F566" s="3">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="G566" s="1"/>
+      <c r="H566" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="567" spans="1:8">
+      <c r="A567" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B567" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C567" s="8">
+        <v>160</v>
+      </c>
+      <c r="D567" s="4">
+        <v>29.823340469051601</v>
+      </c>
+      <c r="E567" s="6">
+        <v>20</v>
+      </c>
+      <c r="F567" s="3">
+        <f t="shared" si="11"/>
+        <v>23.85867237524128</v>
+      </c>
+      <c r="G567" s="1"/>
+      <c r="H567" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="568" spans="1:8">
+      <c r="A568" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B568" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C568" s="8">
+        <v>136</v>
+      </c>
+      <c r="D568" s="4">
+        <v>62.676300164771803</v>
+      </c>
+      <c r="E568" s="6">
+        <v>20</v>
+      </c>
+      <c r="F568" s="3">
+        <f t="shared" si="11"/>
+        <v>50.141040131817441</v>
+      </c>
+      <c r="G568" s="1"/>
+      <c r="H568" s="7"/>
+    </row>
+    <row r="569" spans="1:8">
+      <c r="A569" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B569" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C569" s="8">
+        <v>56</v>
+      </c>
+      <c r="D569" s="4">
+        <v>31.9272796610169</v>
+      </c>
+      <c r="E569" s="6">
+        <v>20</v>
+      </c>
+      <c r="F569" s="3">
+        <f t="shared" si="11"/>
+        <v>25.541823728813519</v>
+      </c>
+      <c r="G569" s="1"/>
+      <c r="H569" s="7"/>
+    </row>
+    <row r="570" spans="1:8">
+      <c r="A570" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B570" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C570" s="8">
+        <v>24</v>
+      </c>
+      <c r="D570" s="4">
+        <v>350.49523185483901</v>
+      </c>
+      <c r="E570" s="6">
+        <v>20</v>
+      </c>
+      <c r="F570" s="3">
+        <f t="shared" si="11"/>
+        <v>280.39618548387119</v>
+      </c>
+      <c r="G570" s="1"/>
+      <c r="H570" s="7"/>
+    </row>
+    <row r="571" spans="1:8">
+      <c r="A571" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="B571" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C571" s="8">
+        <v>24</v>
+      </c>
+      <c r="D571" s="4">
+        <v>226.51426704545401</v>
+      </c>
+      <c r="E571" s="6">
+        <v>20</v>
+      </c>
+      <c r="F571" s="3">
+        <f t="shared" ref="F571:F578" si="12">D571-(D571*E571)/100</f>
+        <v>181.2114136363632</v>
+      </c>
+      <c r="G571" s="1"/>
+      <c r="H571" s="7"/>
+    </row>
+    <row r="572" spans="1:8">
+      <c r="A572" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B572" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C572" s="8">
+        <v>8</v>
+      </c>
+      <c r="D572" s="4">
+        <v>39.116093220339003</v>
+      </c>
+      <c r="E572" s="6">
+        <v>20</v>
+      </c>
+      <c r="F572" s="3">
+        <f t="shared" si="12"/>
+        <v>31.292874576271203</v>
+      </c>
+      <c r="G572" s="1"/>
+      <c r="H572" s="7"/>
+    </row>
+    <row r="573" spans="1:8">
+      <c r="A573" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B573" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C573" s="8">
+        <v>83</v>
+      </c>
+      <c r="D573" s="4">
+        <v>50.484707470537401</v>
+      </c>
+      <c r="E573" s="6">
+        <v>20</v>
+      </c>
+      <c r="F573" s="3">
+        <f t="shared" si="12"/>
+        <v>40.387765976429918</v>
+      </c>
+      <c r="G573" s="1"/>
+      <c r="H573" s="7"/>
+    </row>
+    <row r="574" spans="1:8">
+      <c r="A574" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B574" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C574" s="20">
+        <v>8</v>
+      </c>
+      <c r="D574" s="4">
+        <v>39.116093220339003</v>
+      </c>
+      <c r="E574" s="6">
+        <v>20</v>
+      </c>
+      <c r="F574" s="3">
+        <f t="shared" si="12"/>
+        <v>31.292874576271203</v>
+      </c>
+      <c r="G574" s="1"/>
+      <c r="H574" s="7"/>
+    </row>
+    <row r="575" spans="1:8">
+      <c r="A575" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="B575" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C575" s="26">
+        <v>144</v>
+      </c>
+      <c r="D575" s="4">
+        <v>28.453307923980599</v>
+      </c>
+      <c r="E575" s="6">
+        <v>20</v>
+      </c>
+      <c r="F575" s="3">
+        <f t="shared" si="12"/>
+        <v>22.762646339184478</v>
+      </c>
+      <c r="G575" s="1"/>
+      <c r="H575" s="7"/>
+    </row>
+    <row r="576" spans="1:8">
+      <c r="A576" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B576" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C576" s="26">
+        <v>124</v>
+      </c>
+      <c r="D576" s="4">
+        <v>27.062690707683899</v>
+      </c>
+      <c r="E576" s="6">
+        <v>20</v>
+      </c>
+      <c r="F576" s="3">
+        <f t="shared" si="12"/>
+        <v>21.650152566147121</v>
+      </c>
+      <c r="G576" s="1"/>
+      <c r="H576" s="1"/>
+    </row>
+    <row r="577" spans="1:8">
+      <c r="A577" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B577" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C577" s="26"/>
+      <c r="D577" s="4"/>
+      <c r="E577" s="6">
+        <v>20</v>
+      </c>
+      <c r="F577" s="3">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G577" s="1"/>
+      <c r="H577" s="1"/>
+    </row>
+    <row r="578" spans="1:8">
+      <c r="A578" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B578" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C578" s="26"/>
+      <c r="D578" s="4"/>
+      <c r="E578" s="6">
+        <v>20</v>
+      </c>
+      <c r="F578" s="3">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G578" s="1"/>
+      <c r="H578" s="1"/>
+    </row>
+    <row r="579" spans="1:8">
+      <c r="A579" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B579" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C579" s="26">
+        <v>24</v>
+      </c>
+      <c r="D579" s="4">
+        <v>55.246318385650198</v>
+      </c>
+      <c r="E579" s="6">
+        <v>20</v>
+      </c>
+      <c r="F579" s="3">
+        <f>D579-(D579*E579)/100</f>
+        <v>44.197054708520156</v>
+      </c>
+      <c r="G579" s="1"/>
+      <c r="H579" s="1"/>
+    </row>
+    <row r="580" spans="1:8">
+      <c r="A580" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B580" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C580" s="8">
+        <v>135</v>
+      </c>
+      <c r="D580" s="11">
+        <v>32.569943283582099</v>
+      </c>
+      <c r="E580" s="12">
+        <v>20</v>
+      </c>
+      <c r="F580" s="13">
+        <f t="shared" ref="F580:F643" si="13">D580-(D580*E580)/100</f>
+        <v>26.055954626865677</v>
+      </c>
+      <c r="G580" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H580" s="15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="581" spans="1:8">
+      <c r="A581" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B581" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C581" s="8">
+        <v>32</v>
+      </c>
+      <c r="D581" s="4">
+        <v>66.758647373338903</v>
+      </c>
+      <c r="E581" s="6">
+        <v>20</v>
+      </c>
+      <c r="F581" s="3">
+        <f t="shared" si="13"/>
+        <v>53.406917898671125</v>
+      </c>
+      <c r="G581" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H581" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="582" spans="1:8">
+      <c r="A582" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B582" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C582" s="8"/>
+      <c r="D582" s="4"/>
+      <c r="E582" s="6">
+        <v>20</v>
+      </c>
+      <c r="F582" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G582" s="1"/>
+      <c r="H582" s="7"/>
+    </row>
+    <row r="583" spans="1:8">
+      <c r="A583" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B583" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C583" s="8">
+        <v>168</v>
+      </c>
+      <c r="D583" s="4">
+        <v>31.530817164179101</v>
+      </c>
+      <c r="E583" s="6">
+        <v>20</v>
+      </c>
+      <c r="F583" s="3">
+        <f t="shared" si="13"/>
+        <v>25.224653731343281</v>
+      </c>
+      <c r="G583" s="1"/>
+      <c r="H583" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="584" spans="1:8">
+      <c r="A584" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B584" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C584" s="8">
+        <v>112</v>
+      </c>
+      <c r="D584" s="4">
+        <v>64.374991279069803</v>
+      </c>
+      <c r="E584" s="6">
+        <v>20</v>
+      </c>
+      <c r="F584" s="3">
+        <f t="shared" si="13"/>
+        <v>51.49999302325584</v>
+      </c>
+      <c r="G584" s="1"/>
+      <c r="H584" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="585" spans="1:8">
+      <c r="A585" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B585" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C585" s="8">
+        <v>152</v>
+      </c>
+      <c r="D585" s="4">
+        <v>29.974938469837699</v>
+      </c>
+      <c r="E585" s="6">
+        <v>20</v>
+      </c>
+      <c r="F585" s="3">
+        <f t="shared" si="13"/>
+        <v>23.979950775870158</v>
+      </c>
+      <c r="G585" s="1"/>
+      <c r="H585" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="586" spans="1:8">
+      <c r="A586" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B586" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C586" s="8">
+        <v>160</v>
+      </c>
+      <c r="D586" s="4">
+        <v>33.366855427807501</v>
+      </c>
+      <c r="E586" s="6">
+        <v>20</v>
+      </c>
+      <c r="F586" s="3">
+        <f t="shared" si="13"/>
+        <v>26.693484342246002</v>
+      </c>
+      <c r="G586" s="1"/>
+      <c r="H586" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="587" spans="1:8">
+      <c r="A587" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B587" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C587" s="8">
+        <v>192</v>
+      </c>
+      <c r="D587" s="4">
+        <v>36.709279166666697</v>
+      </c>
+      <c r="E587" s="6">
+        <v>20</v>
+      </c>
+      <c r="F587" s="3">
+        <f t="shared" si="13"/>
+        <v>29.367423333333356</v>
+      </c>
+      <c r="G587" s="1"/>
+      <c r="H587" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="588" spans="1:8">
+      <c r="A588" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B588" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C588" s="8">
+        <v>152</v>
+      </c>
+      <c r="D588" s="4">
+        <v>39.802379807692297</v>
+      </c>
+      <c r="E588" s="6">
+        <v>20</v>
+      </c>
+      <c r="F588" s="3">
+        <f t="shared" si="13"/>
+        <v>31.841903846153837</v>
+      </c>
+      <c r="G588" s="1"/>
+      <c r="H588" s="7"/>
+    </row>
+    <row r="589" spans="1:8">
+      <c r="A589" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B589" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C589" s="8">
+        <v>136</v>
+      </c>
+      <c r="D589" s="4">
+        <v>34.0075820776974</v>
+      </c>
+      <c r="E589" s="6">
+        <v>20</v>
+      </c>
+      <c r="F589" s="3">
+        <f t="shared" si="13"/>
+        <v>27.206065662157918</v>
+      </c>
+      <c r="G589" s="1"/>
+      <c r="H589" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="590" spans="1:8">
+      <c r="A590" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B590" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C590" s="8">
+        <v>151</v>
+      </c>
+      <c r="D590" s="4">
+        <v>56.1774309696156</v>
+      </c>
+      <c r="E590" s="6">
+        <v>20</v>
+      </c>
+      <c r="F590" s="3">
+        <f t="shared" si="13"/>
+        <v>44.941944775692477</v>
+      </c>
+      <c r="G590" s="1"/>
+      <c r="H590" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="591" spans="1:8">
+      <c r="A591" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B591" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C591" s="8">
+        <v>199</v>
+      </c>
+      <c r="D591" s="4">
+        <v>54.628285714285703</v>
+      </c>
+      <c r="E591" s="6">
+        <v>20</v>
+      </c>
+      <c r="F591" s="3">
+        <f t="shared" si="13"/>
+        <v>43.702628571428562</v>
+      </c>
+      <c r="G591" s="1"/>
+      <c r="H591" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="592" spans="1:8">
+      <c r="A592" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B592" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C592" s="8">
+        <v>144</v>
+      </c>
+      <c r="D592" s="4">
+        <v>45.963287985588998</v>
+      </c>
+      <c r="E592" s="6">
+        <v>20</v>
+      </c>
+      <c r="F592" s="3">
+        <f t="shared" si="13"/>
+        <v>36.770630388471197</v>
+      </c>
+      <c r="G592" s="1"/>
+      <c r="H592" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="593" spans="1:8">
+      <c r="A593" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B593" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C593" s="8">
+        <v>152</v>
+      </c>
+      <c r="D593" s="4">
+        <v>29.974938469837699</v>
+      </c>
+      <c r="E593" s="6">
+        <v>20</v>
+      </c>
+      <c r="F593" s="3">
+        <f t="shared" si="13"/>
+        <v>23.979950775870158</v>
+      </c>
+      <c r="G593" s="1"/>
+      <c r="H593" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="594" spans="1:8">
+      <c r="A594" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B594" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C594" s="8">
+        <v>120</v>
+      </c>
+      <c r="D594" s="4">
+        <v>64.374991279069803</v>
+      </c>
+      <c r="E594" s="6">
+        <v>20</v>
+      </c>
+      <c r="F594" s="3">
+        <f t="shared" si="13"/>
+        <v>51.49999302325584</v>
+      </c>
+      <c r="G594" s="1"/>
+      <c r="H594" s="7"/>
+    </row>
+    <row r="595" spans="1:8">
+      <c r="A595" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B595" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C595" s="8">
+        <v>176</v>
+      </c>
+      <c r="D595" s="4">
+        <v>40.9208262195122</v>
+      </c>
+      <c r="E595" s="6">
+        <v>20</v>
+      </c>
+      <c r="F595" s="3">
+        <f t="shared" si="13"/>
+        <v>32.736660975609759</v>
+      </c>
+      <c r="G595" s="1"/>
+      <c r="H595" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="596" spans="1:8">
+      <c r="A596" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B596" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C596" s="8">
+        <v>176</v>
+      </c>
+      <c r="D596" s="4">
+        <v>42.457833333333298</v>
+      </c>
+      <c r="E596" s="6">
+        <v>20</v>
+      </c>
+      <c r="F596" s="3">
+        <f t="shared" si="13"/>
+        <v>33.966266666666641</v>
+      </c>
+      <c r="G596" s="1"/>
+      <c r="H596" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="597" spans="1:8">
+      <c r="A597" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B597" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C597" s="8">
+        <v>144</v>
+      </c>
+      <c r="D597" s="4">
+        <v>31.229776295605301</v>
+      </c>
+      <c r="E597" s="6">
+        <v>20</v>
+      </c>
+      <c r="F597" s="3">
+        <f t="shared" si="13"/>
+        <v>24.98382103648424</v>
+      </c>
+      <c r="G597" s="1"/>
+      <c r="H597" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="598" spans="1:8">
+      <c r="A598" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B598" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C598" s="8">
+        <v>120</v>
+      </c>
+      <c r="D598" s="4">
+        <v>45.193713573232301</v>
+      </c>
+      <c r="E598" s="6">
+        <v>20</v>
+      </c>
+      <c r="F598" s="3">
+        <f t="shared" si="13"/>
+        <v>36.154970858585841</v>
+      </c>
+      <c r="G598" s="1"/>
+      <c r="H598" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="599" spans="1:8">
+      <c r="A599" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B599" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C599" s="8">
+        <v>148</v>
+      </c>
+      <c r="D599" s="4">
+        <v>45.9833427159992</v>
+      </c>
+      <c r="E599" s="6">
+        <v>20</v>
+      </c>
+      <c r="F599" s="3">
+        <f t="shared" si="13"/>
+        <v>36.786674172799358</v>
+      </c>
+      <c r="G599" s="1"/>
+      <c r="H599" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="600" spans="1:8">
+      <c r="A600" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B600" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C600" s="8">
+        <v>112</v>
+      </c>
+      <c r="D600" s="4">
+        <v>49.117546875000002</v>
+      </c>
+      <c r="E600" s="6">
+        <v>20</v>
+      </c>
+      <c r="F600" s="3">
+        <f t="shared" si="13"/>
+        <v>39.294037500000002</v>
+      </c>
+      <c r="G600" s="1"/>
+      <c r="H600" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="601" spans="1:8">
+      <c r="A601" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B601" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C601" s="8">
+        <v>148</v>
+      </c>
+      <c r="D601" s="4">
+        <v>43.883568071399203</v>
+      </c>
+      <c r="E601" s="6">
+        <v>20</v>
+      </c>
+      <c r="F601" s="3">
+        <f t="shared" si="13"/>
+        <v>35.106854457119361</v>
+      </c>
+      <c r="G601" s="1"/>
+      <c r="H601" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="602" spans="1:8">
+      <c r="A602" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B602" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C602" s="8">
+        <v>160</v>
+      </c>
+      <c r="D602" s="4">
+        <v>39.855445859792802</v>
+      </c>
+      <c r="E602" s="6">
+        <v>20</v>
+      </c>
+      <c r="F602" s="3">
+        <f t="shared" si="13"/>
+        <v>31.884356687834241</v>
+      </c>
+      <c r="G602" s="1"/>
+      <c r="H602" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="603" spans="1:8">
+      <c r="A603" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B603" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C603" s="8">
+        <v>168</v>
+      </c>
+      <c r="D603" s="4">
+        <v>47.282472118081003</v>
+      </c>
+      <c r="E603" s="6">
+        <v>20</v>
+      </c>
+      <c r="F603" s="3">
+        <f t="shared" si="13"/>
+        <v>37.825977694464804</v>
+      </c>
+      <c r="G603" s="1"/>
+      <c r="H603" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="604" spans="1:8">
+      <c r="A604" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B604" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C604" s="8">
+        <v>16</v>
+      </c>
+      <c r="D604" s="4">
+        <v>72.014428571428596</v>
+      </c>
+      <c r="E604" s="6">
+        <v>20</v>
+      </c>
+      <c r="F604" s="3">
+        <f t="shared" si="13"/>
+        <v>57.611542857142879</v>
+      </c>
+      <c r="G604" s="1"/>
+      <c r="H604" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="605" spans="1:8">
+      <c r="A605" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B605" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C605" s="8"/>
+      <c r="D605" s="4"/>
+      <c r="E605" s="6">
+        <v>20</v>
+      </c>
+      <c r="F605" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G605" s="1"/>
+      <c r="H605" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="606" spans="1:8">
+      <c r="A606" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B606" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C606" s="8">
+        <v>168</v>
+      </c>
+      <c r="D606" s="4">
+        <v>31.530817164179101</v>
+      </c>
+      <c r="E606" s="6">
+        <v>20</v>
+      </c>
+      <c r="F606" s="3">
+        <f t="shared" si="13"/>
+        <v>25.224653731343281</v>
+      </c>
+      <c r="G606" s="1"/>
+      <c r="H606" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="607" spans="1:8">
+      <c r="A607" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B607" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C607" s="8">
+        <v>133</v>
+      </c>
+      <c r="D607" s="4">
+        <v>48.468821146473502</v>
+      </c>
+      <c r="E607" s="6">
+        <v>20</v>
+      </c>
+      <c r="F607" s="3">
+        <f t="shared" si="13"/>
+        <v>38.775056917178802</v>
+      </c>
+      <c r="G607" s="1"/>
+      <c r="H607" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="608" spans="1:8">
+      <c r="A608" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B608" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C608" s="8">
+        <v>16</v>
+      </c>
+      <c r="D608" s="4">
+        <v>64.374991279069803</v>
+      </c>
+      <c r="E608" s="6">
+        <v>20</v>
+      </c>
+      <c r="F608" s="3">
+        <f t="shared" si="13"/>
+        <v>51.49999302325584</v>
+      </c>
+      <c r="G608" s="1"/>
+      <c r="H608" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="609" spans="1:8">
+      <c r="A609" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B609" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C609" s="8">
+        <v>168</v>
+      </c>
+      <c r="D609" s="4">
+        <v>45.8907234848485</v>
+      </c>
+      <c r="E609" s="6">
+        <v>20</v>
+      </c>
+      <c r="F609" s="3">
+        <f t="shared" si="13"/>
+        <v>36.712578787878797</v>
+      </c>
+      <c r="G609" s="1"/>
+      <c r="H609" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="610" spans="1:8">
+      <c r="A610" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B610" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C610" s="8">
+        <v>168</v>
+      </c>
+      <c r="D610" s="4">
+        <v>44.993664730104399</v>
+      </c>
+      <c r="E610" s="6">
+        <v>20</v>
+      </c>
+      <c r="F610" s="3">
+        <f t="shared" si="13"/>
+        <v>35.994931784083519</v>
+      </c>
+      <c r="G610" s="1"/>
+      <c r="H610" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="611" spans="1:8">
+      <c r="A611" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B611" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C611" s="8">
+        <v>152</v>
+      </c>
+      <c r="D611" s="4">
+        <v>91.7073898096248</v>
+      </c>
+      <c r="E611" s="6">
+        <v>20</v>
+      </c>
+      <c r="F611" s="3">
+        <f t="shared" si="13"/>
+        <v>73.365911847699834</v>
+      </c>
+      <c r="G611" s="1"/>
+      <c r="H611" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="612" spans="1:8">
+      <c r="A612" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B612" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C612" s="8">
+        <v>200</v>
+      </c>
+      <c r="D612" s="4">
+        <v>33.869991249999998</v>
+      </c>
+      <c r="E612" s="6">
+        <v>20</v>
+      </c>
+      <c r="F612" s="3">
+        <f t="shared" si="13"/>
+        <v>27.095993</v>
+      </c>
+      <c r="G612" s="1"/>
+      <c r="H612" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="613" spans="1:8">
+      <c r="A613" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B613" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C613" s="8">
+        <v>160</v>
+      </c>
+      <c r="D613" s="4">
+        <v>75.671888476493393</v>
+      </c>
+      <c r="E613" s="6">
+        <v>20</v>
+      </c>
+      <c r="F613" s="3">
+        <f t="shared" si="13"/>
+        <v>60.537510781194712</v>
+      </c>
+      <c r="G613" s="1"/>
+      <c r="H613" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="614" spans="1:8">
+      <c r="A614" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B614" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C614" s="8">
+        <v>24</v>
+      </c>
+      <c r="D614" s="4">
+        <v>64.374991279069803</v>
+      </c>
+      <c r="E614" s="6">
+        <v>20</v>
+      </c>
+      <c r="F614" s="3">
+        <f t="shared" si="13"/>
+        <v>51.49999302325584</v>
+      </c>
+      <c r="G614" s="1"/>
+      <c r="H614" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="615" spans="1:8">
+      <c r="A615" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B615" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C615" s="8">
+        <v>24</v>
+      </c>
+      <c r="D615" s="4">
+        <v>72.014428571428596</v>
+      </c>
+      <c r="E615" s="6">
+        <v>20</v>
+      </c>
+      <c r="F615" s="3">
+        <f t="shared" si="13"/>
+        <v>57.611542857142879</v>
+      </c>
+      <c r="G615" s="1"/>
+      <c r="H615" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="616" spans="1:8">
+      <c r="A616" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B616" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C616" s="8">
+        <v>168</v>
+      </c>
+      <c r="D616" s="4">
+        <v>31.530817164179101</v>
+      </c>
+      <c r="E616" s="6">
+        <v>20</v>
+      </c>
+      <c r="F616" s="3">
+        <f t="shared" si="13"/>
+        <v>25.224653731343281</v>
+      </c>
+      <c r="G616" s="1"/>
+      <c r="H616" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="617" spans="1:8">
+      <c r="A617" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B617" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C617" s="8">
+        <v>143</v>
+      </c>
+      <c r="D617" s="4">
+        <v>40.2840582191781</v>
+      </c>
+      <c r="E617" s="6">
+        <v>20</v>
+      </c>
+      <c r="F617" s="3">
+        <f t="shared" si="13"/>
+        <v>32.227246575342477</v>
+      </c>
+      <c r="G617" s="1"/>
+      <c r="H617" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="618" spans="1:8">
+      <c r="A618" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B618" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C618" s="8">
+        <v>168</v>
+      </c>
+      <c r="D618" s="4">
+        <v>36.1385890314547</v>
+      </c>
+      <c r="E618" s="6">
+        <v>20</v>
+      </c>
+      <c r="F618" s="3">
+        <f t="shared" si="13"/>
+        <v>28.91087122516376</v>
+      </c>
+      <c r="G618" s="1"/>
+      <c r="H618" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="619" spans="1:8">
+      <c r="A619" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B619" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C619" s="8">
+        <v>184</v>
+      </c>
+      <c r="D619" s="4">
+        <v>40.175800000000002</v>
+      </c>
+      <c r="E619" s="6">
+        <v>20</v>
+      </c>
+      <c r="F619" s="3">
+        <f t="shared" si="13"/>
+        <v>32.140640000000005</v>
+      </c>
+      <c r="G619" s="1"/>
+      <c r="H619" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="620" spans="1:8">
+      <c r="A620" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B620" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C620" s="8">
+        <v>40</v>
+      </c>
+      <c r="D620" s="4">
+        <v>69.358899190199296</v>
+      </c>
+      <c r="E620" s="6">
+        <v>20</v>
+      </c>
+      <c r="F620" s="3">
+        <f t="shared" si="13"/>
+        <v>55.487119352159439</v>
+      </c>
+      <c r="G620" s="1"/>
+      <c r="H620" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="621" spans="1:8">
+      <c r="A621" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B621" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C621" s="8">
+        <v>112</v>
+      </c>
+      <c r="D621" s="4">
+        <v>33.790650468504303</v>
+      </c>
+      <c r="E621" s="6">
+        <v>20</v>
+      </c>
+      <c r="F621" s="3">
+        <f t="shared" si="13"/>
+        <v>27.032520374803443</v>
+      </c>
+      <c r="G621" s="1"/>
+      <c r="H621" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="622" spans="1:8">
+      <c r="A622" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B622" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C622" s="8"/>
+      <c r="D622" s="4"/>
+      <c r="E622" s="6">
+        <v>20</v>
+      </c>
+      <c r="F622" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G622" s="1"/>
+      <c r="H622" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="623" spans="1:8">
+      <c r="A623" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B623" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C623" s="8">
+        <v>80</v>
+      </c>
+      <c r="D623" s="4">
+        <v>111.66268035752201</v>
+      </c>
+      <c r="E623" s="6">
+        <v>20</v>
+      </c>
+      <c r="F623" s="3">
+        <f t="shared" si="13"/>
+        <v>89.3301442860176</v>
+      </c>
+      <c r="G623" s="1"/>
+      <c r="H623" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="624" spans="1:8">
+      <c r="A624" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B624" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C624" s="8">
+        <v>152</v>
+      </c>
+      <c r="D624" s="4">
+        <v>91.7073898096248</v>
+      </c>
+      <c r="E624" s="6">
+        <v>20</v>
+      </c>
+      <c r="F624" s="3">
+        <f t="shared" si="13"/>
+        <v>73.365911847699834</v>
+      </c>
+      <c r="G624" s="1"/>
+      <c r="H624" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="625" spans="1:8">
+      <c r="A625" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B625" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C625" s="8"/>
+      <c r="D625" s="4"/>
+      <c r="E625" s="6">
+        <v>20</v>
+      </c>
+      <c r="F625" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G625" s="1"/>
+      <c r="H625" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="626" spans="1:8">
+      <c r="A626" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B626" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C626" s="8"/>
+      <c r="D626" s="4"/>
+      <c r="E626" s="6">
+        <v>20</v>
+      </c>
+      <c r="F626" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G626" s="1"/>
+      <c r="H626" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="627" spans="1:8">
+      <c r="A627" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B627" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C627" s="8">
+        <v>8</v>
+      </c>
+      <c r="D627" s="4">
+        <v>21.555375000000002</v>
+      </c>
+      <c r="E627" s="6">
+        <v>20</v>
+      </c>
+      <c r="F627" s="3">
+        <f t="shared" si="13"/>
+        <v>17.244300000000003</v>
+      </c>
+      <c r="G627" s="1"/>
+      <c r="H627" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="628" spans="1:8">
+      <c r="A628" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B628" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C628" s="8"/>
+      <c r="D628" s="4"/>
+      <c r="E628" s="6">
+        <v>20</v>
+      </c>
+      <c r="F628" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G628" s="1"/>
+      <c r="H628" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="629" spans="1:8">
+      <c r="A629" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B629" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C629" s="8">
+        <v>168</v>
+      </c>
+      <c r="D629" s="4">
+        <v>42.752038640873003</v>
+      </c>
+      <c r="E629" s="6">
+        <v>20</v>
+      </c>
+      <c r="F629" s="3">
+        <f t="shared" si="13"/>
+        <v>34.201630912698405</v>
+      </c>
+      <c r="G629" s="1"/>
+      <c r="H629" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="630" spans="1:8">
+      <c r="A630" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B630" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C630" s="8">
+        <v>8</v>
+      </c>
+      <c r="D630" s="4">
+        <v>44.180250000000001</v>
+      </c>
+      <c r="E630" s="6">
+        <v>20</v>
+      </c>
+      <c r="F630" s="3">
+        <f t="shared" si="13"/>
+        <v>35.344200000000001</v>
+      </c>
+      <c r="G630" s="1"/>
+      <c r="H630" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="631" spans="1:8">
+      <c r="A631" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B631" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C631" s="8">
+        <v>104</v>
+      </c>
+      <c r="D631" s="4">
+        <v>40.9208262195122</v>
+      </c>
+      <c r="E631" s="6">
+        <v>20</v>
+      </c>
+      <c r="F631" s="3">
+        <f t="shared" si="13"/>
+        <v>32.736660975609759</v>
+      </c>
+      <c r="G631" s="1"/>
+      <c r="H631" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="632" spans="1:8">
+      <c r="A632" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B632" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C632" s="8"/>
+      <c r="D632" s="4"/>
+      <c r="E632" s="6">
+        <v>20</v>
+      </c>
+      <c r="F632" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G632" s="1"/>
+      <c r="H632" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="633" spans="1:8">
+      <c r="A633" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B633" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C633" s="8">
+        <v>8</v>
+      </c>
+      <c r="D633" s="4">
+        <v>21.555375000000002</v>
+      </c>
+      <c r="E633" s="6">
+        <v>20</v>
+      </c>
+      <c r="F633" s="3">
+        <f t="shared" si="13"/>
+        <v>17.244300000000003</v>
+      </c>
+      <c r="G633" s="1"/>
+      <c r="H633" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="634" spans="1:8">
+      <c r="A634" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B634" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C634" s="8">
+        <v>108</v>
+      </c>
+      <c r="D634" s="4">
+        <v>29.890958877995601</v>
+      </c>
+      <c r="E634" s="6">
+        <v>20</v>
+      </c>
+      <c r="F634" s="3">
+        <f t="shared" si="13"/>
+        <v>23.912767102396479</v>
+      </c>
+      <c r="G634" s="1"/>
+      <c r="H634" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="635" spans="1:8">
+      <c r="A635" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B635" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C635" s="8">
+        <v>152</v>
+      </c>
+      <c r="D635" s="4">
+        <v>45.453582236842102</v>
+      </c>
+      <c r="E635" s="6">
+        <v>20</v>
+      </c>
+      <c r="F635" s="3">
+        <f t="shared" si="13"/>
+        <v>36.36286578947368</v>
+      </c>
+      <c r="G635" s="1"/>
+      <c r="H635" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="636" spans="1:8">
+      <c r="A636" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B636" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C636" s="8">
+        <v>152</v>
+      </c>
+      <c r="D636" s="4">
+        <v>55.974312500000003</v>
+      </c>
+      <c r="E636" s="6">
+        <v>20</v>
+      </c>
+      <c r="F636" s="3">
+        <f t="shared" si="13"/>
+        <v>44.779450000000004</v>
+      </c>
+      <c r="G636" s="1"/>
+      <c r="H636" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="637" spans="1:8">
+      <c r="A637" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B637" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C637" s="8">
+        <v>152</v>
+      </c>
+      <c r="D637" s="4">
+        <v>55.974312500000003</v>
+      </c>
+      <c r="E637" s="6">
+        <v>20</v>
+      </c>
+      <c r="F637" s="3">
+        <f t="shared" si="13"/>
+        <v>44.779450000000004</v>
+      </c>
+      <c r="G637" s="1"/>
+      <c r="H637" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="638" spans="1:8">
+      <c r="A638" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B638" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C638" s="8">
+        <v>31</v>
+      </c>
+      <c r="D638" s="4">
+        <v>62.174122280570103</v>
+      </c>
+      <c r="E638" s="6">
+        <v>20</v>
+      </c>
+      <c r="F638" s="3">
+        <f t="shared" si="13"/>
+        <v>49.739297824456081</v>
+      </c>
+      <c r="G638" s="1"/>
+      <c r="H638" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="639" spans="1:8">
+      <c r="A639" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B639" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C639" s="8">
+        <v>184</v>
+      </c>
+      <c r="D639" s="4">
+        <v>41.455352356177102</v>
+      </c>
+      <c r="E639" s="6">
+        <v>20</v>
+      </c>
+      <c r="F639" s="3">
+        <f t="shared" si="13"/>
+        <v>33.16428188494168</v>
+      </c>
+      <c r="G639" s="1"/>
+      <c r="H639" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="640" spans="1:8">
+      <c r="A640" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B640" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C640" s="8">
+        <v>104</v>
+      </c>
+      <c r="D640" s="4">
+        <v>99.887291645690794</v>
+      </c>
+      <c r="E640" s="6">
+        <v>20</v>
+      </c>
+      <c r="F640" s="3">
+        <f t="shared" si="13"/>
+        <v>79.909833316552636</v>
+      </c>
+      <c r="G640" s="1"/>
+      <c r="H640" s="7"/>
+    </row>
+    <row r="641" spans="1:8">
+      <c r="A641" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B641" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C641" s="8">
+        <v>143</v>
+      </c>
+      <c r="D641" s="4">
+        <v>40.2840582191781</v>
+      </c>
+      <c r="E641" s="6">
+        <v>20</v>
+      </c>
+      <c r="F641" s="3">
+        <f t="shared" si="13"/>
+        <v>32.227246575342477</v>
+      </c>
+      <c r="G641" s="1"/>
+      <c r="H641" s="7"/>
+    </row>
+    <row r="642" spans="1:8">
+      <c r="A642" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B642" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C642" s="8"/>
+      <c r="D642" s="4"/>
+      <c r="E642" s="6">
+        <v>20</v>
+      </c>
+      <c r="F642" s="3">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="G642" s="1"/>
+      <c r="H642" s="7"/>
+    </row>
+    <row r="643" spans="1:8">
+      <c r="A643" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="B643" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C643" s="8">
+        <v>8</v>
+      </c>
+      <c r="D643" s="4">
+        <v>39.802379807692297</v>
+      </c>
+      <c r="E643" s="6">
+        <v>20</v>
+      </c>
+      <c r="F643" s="3">
+        <f t="shared" si="13"/>
+        <v>31.841903846153837</v>
+      </c>
+      <c r="G643" s="1"/>
+      <c r="H643" s="7"/>
+    </row>
+    <row r="644" spans="1:8">
+      <c r="A644" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B644" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C644" s="8">
+        <v>32</v>
+      </c>
+      <c r="D644" s="4">
+        <v>54.887776609492498</v>
+      </c>
+      <c r="E644" s="6">
+        <v>20</v>
+      </c>
+      <c r="F644" s="3">
+        <f t="shared" ref="F644:F651" si="14">D644-(D644*E644)/100</f>
+        <v>43.910221287593998</v>
+      </c>
+      <c r="G644" s="1"/>
+      <c r="H644" s="7"/>
+    </row>
+    <row r="645" spans="1:8">
+      <c r="A645" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B645" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C645" s="8">
+        <v>152</v>
+      </c>
+      <c r="D645" s="4">
+        <v>49.890653224368798</v>
+      </c>
+      <c r="E645" s="6">
+        <v>20</v>
+      </c>
+      <c r="F645" s="3">
+        <f t="shared" si="14"/>
+        <v>39.91252257949504</v>
+      </c>
+      <c r="G645" s="1"/>
+      <c r="H645" s="7"/>
+    </row>
+    <row r="646" spans="1:8">
+      <c r="A646" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B646" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C646" s="20"/>
+      <c r="D646" s="4"/>
+      <c r="E646" s="6">
+        <v>20</v>
+      </c>
+      <c r="F646" s="3">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="G646" s="1"/>
+      <c r="H646" s="7"/>
+    </row>
+    <row r="647" spans="1:8">
+      <c r="A647" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="B647" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C647" s="26">
+        <v>152</v>
+      </c>
+      <c r="D647" s="4">
+        <v>33.735907565789503</v>
+      </c>
+      <c r="E647" s="6">
+        <v>20</v>
+      </c>
+      <c r="F647" s="3">
+        <f t="shared" si="14"/>
+        <v>26.988726052631602</v>
+      </c>
+      <c r="G647" s="1"/>
+      <c r="H647" s="7"/>
+    </row>
+    <row r="648" spans="1:8">
+      <c r="A648" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B648" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C648" s="26">
+        <v>146</v>
+      </c>
+      <c r="D648" s="4">
+        <v>35.337836316328499</v>
+      </c>
+      <c r="E648" s="6">
+        <v>20</v>
+      </c>
+      <c r="F648" s="3">
+        <f t="shared" si="14"/>
+        <v>28.270269053062798</v>
+      </c>
+      <c r="G648" s="1"/>
+      <c r="H648" s="1"/>
+    </row>
+    <row r="649" spans="1:8">
+      <c r="A649" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B649" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C649" s="26"/>
+      <c r="D649" s="4"/>
+      <c r="E649" s="6">
+        <v>20</v>
+      </c>
+      <c r="F649" s="3">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="G649" s="1"/>
+      <c r="H649" s="1"/>
+    </row>
+    <row r="650" spans="1:8">
+      <c r="A650" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B650" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C650" s="26"/>
+      <c r="D650" s="4"/>
+      <c r="E650" s="6">
+        <v>20</v>
+      </c>
+      <c r="F650" s="3">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="G650" s="1"/>
+      <c r="H650" s="1"/>
+    </row>
+    <row r="651" spans="1:8">
+      <c r="A651" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B651" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C651" s="26"/>
+      <c r="D651" s="4"/>
+      <c r="E651" s="6">
+        <v>20</v>
+      </c>
+      <c r="F651" s="3">
+        <f>D651-(D651*E651)/100</f>
+        <v>0</v>
+      </c>
+      <c r="G651" s="1"/>
+      <c r="H651" s="1"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G507">
+  <autoFilter ref="A1:G651">
     <filterColumn colId="0"/>
     <filterColumn colId="1"/>
   </autoFilter>
@@ -13868,6 +17320,122 @@
     <hyperlink ref="H491" r:id="rId420"/>
     <hyperlink ref="H492" r:id="rId421"/>
     <hyperlink ref="H493" r:id="rId422"/>
+    <hyperlink ref="G508" r:id="rId423"/>
+    <hyperlink ref="H508" r:id="rId424"/>
+    <hyperlink ref="H509" r:id="rId425"/>
+    <hyperlink ref="H511" r:id="rId426"/>
+    <hyperlink ref="H512" r:id="rId427"/>
+    <hyperlink ref="H513" r:id="rId428"/>
+    <hyperlink ref="H514" r:id="rId429"/>
+    <hyperlink ref="H515" r:id="rId430"/>
+    <hyperlink ref="H517" r:id="rId431"/>
+    <hyperlink ref="H518" r:id="rId432"/>
+    <hyperlink ref="H519" r:id="rId433"/>
+    <hyperlink ref="H520" r:id="rId434"/>
+    <hyperlink ref="H521" r:id="rId435"/>
+    <hyperlink ref="H523" r:id="rId436"/>
+    <hyperlink ref="H524" r:id="rId437"/>
+    <hyperlink ref="H525" r:id="rId438"/>
+    <hyperlink ref="H526" r:id="rId439"/>
+    <hyperlink ref="H527" r:id="rId440"/>
+    <hyperlink ref="H528" r:id="rId441"/>
+    <hyperlink ref="H529" r:id="rId442"/>
+    <hyperlink ref="H530" r:id="rId443"/>
+    <hyperlink ref="H531" r:id="rId444"/>
+    <hyperlink ref="H532" r:id="rId445"/>
+    <hyperlink ref="H533" r:id="rId446"/>
+    <hyperlink ref="H534" r:id="rId447"/>
+    <hyperlink ref="H535" r:id="rId448"/>
+    <hyperlink ref="H536" r:id="rId449"/>
+    <hyperlink ref="H537" r:id="rId450"/>
+    <hyperlink ref="H538" r:id="rId451"/>
+    <hyperlink ref="H539" r:id="rId452"/>
+    <hyperlink ref="H540" r:id="rId453"/>
+    <hyperlink ref="H541" r:id="rId454"/>
+    <hyperlink ref="H542" r:id="rId455"/>
+    <hyperlink ref="H543" r:id="rId456"/>
+    <hyperlink ref="H544" r:id="rId457"/>
+    <hyperlink ref="H545" r:id="rId458"/>
+    <hyperlink ref="H546" r:id="rId459"/>
+    <hyperlink ref="H547" r:id="rId460"/>
+    <hyperlink ref="H548" r:id="rId461"/>
+    <hyperlink ref="H549" r:id="rId462"/>
+    <hyperlink ref="H550" r:id="rId463"/>
+    <hyperlink ref="H551" r:id="rId464"/>
+    <hyperlink ref="H552" r:id="rId465"/>
+    <hyperlink ref="H553" r:id="rId466"/>
+    <hyperlink ref="H554" r:id="rId467"/>
+    <hyperlink ref="H555" r:id="rId468"/>
+    <hyperlink ref="H556" r:id="rId469"/>
+    <hyperlink ref="H557" r:id="rId470"/>
+    <hyperlink ref="H558" r:id="rId471"/>
+    <hyperlink ref="H559" r:id="rId472"/>
+    <hyperlink ref="H560" r:id="rId473"/>
+    <hyperlink ref="H561" r:id="rId474"/>
+    <hyperlink ref="H562" r:id="rId475"/>
+    <hyperlink ref="H563" r:id="rId476"/>
+    <hyperlink ref="H564" r:id="rId477"/>
+    <hyperlink ref="H565" r:id="rId478"/>
+    <hyperlink ref="H566" r:id="rId479"/>
+    <hyperlink ref="H567" r:id="rId480"/>
+    <hyperlink ref="G580" r:id="rId481"/>
+    <hyperlink ref="H580" r:id="rId482"/>
+    <hyperlink ref="H581" r:id="rId483"/>
+    <hyperlink ref="H583" r:id="rId484"/>
+    <hyperlink ref="H584" r:id="rId485"/>
+    <hyperlink ref="H585" r:id="rId486"/>
+    <hyperlink ref="H586" r:id="rId487"/>
+    <hyperlink ref="H587" r:id="rId488"/>
+    <hyperlink ref="H589" r:id="rId489"/>
+    <hyperlink ref="H590" r:id="rId490"/>
+    <hyperlink ref="H591" r:id="rId491"/>
+    <hyperlink ref="H592" r:id="rId492"/>
+    <hyperlink ref="H593" r:id="rId493"/>
+    <hyperlink ref="H595" r:id="rId494"/>
+    <hyperlink ref="H596" r:id="rId495"/>
+    <hyperlink ref="H597" r:id="rId496"/>
+    <hyperlink ref="H598" r:id="rId497"/>
+    <hyperlink ref="H599" r:id="rId498"/>
+    <hyperlink ref="H600" r:id="rId499"/>
+    <hyperlink ref="H601" r:id="rId500"/>
+    <hyperlink ref="H602" r:id="rId501"/>
+    <hyperlink ref="H603" r:id="rId502"/>
+    <hyperlink ref="H604" r:id="rId503"/>
+    <hyperlink ref="H605" r:id="rId504"/>
+    <hyperlink ref="H606" r:id="rId505"/>
+    <hyperlink ref="H607" r:id="rId506"/>
+    <hyperlink ref="H608" r:id="rId507"/>
+    <hyperlink ref="H609" r:id="rId508"/>
+    <hyperlink ref="H610" r:id="rId509"/>
+    <hyperlink ref="H611" r:id="rId510"/>
+    <hyperlink ref="H612" r:id="rId511"/>
+    <hyperlink ref="H613" r:id="rId512"/>
+    <hyperlink ref="H614" r:id="rId513"/>
+    <hyperlink ref="H615" r:id="rId514"/>
+    <hyperlink ref="H616" r:id="rId515"/>
+    <hyperlink ref="H617" r:id="rId516"/>
+    <hyperlink ref="H618" r:id="rId517"/>
+    <hyperlink ref="H619" r:id="rId518"/>
+    <hyperlink ref="H620" r:id="rId519"/>
+    <hyperlink ref="H621" r:id="rId520"/>
+    <hyperlink ref="H622" r:id="rId521"/>
+    <hyperlink ref="H623" r:id="rId522"/>
+    <hyperlink ref="H624" r:id="rId523"/>
+    <hyperlink ref="H625" r:id="rId524"/>
+    <hyperlink ref="H626" r:id="rId525"/>
+    <hyperlink ref="H627" r:id="rId526"/>
+    <hyperlink ref="H628" r:id="rId527"/>
+    <hyperlink ref="H629" r:id="rId528"/>
+    <hyperlink ref="H630" r:id="rId529"/>
+    <hyperlink ref="H631" r:id="rId530"/>
+    <hyperlink ref="H632" r:id="rId531"/>
+    <hyperlink ref="H633" r:id="rId532"/>
+    <hyperlink ref="H634" r:id="rId533"/>
+    <hyperlink ref="H635" r:id="rId534"/>
+    <hyperlink ref="H636" r:id="rId535"/>
+    <hyperlink ref="H637" r:id="rId536"/>
+    <hyperlink ref="H638" r:id="rId537"/>
+    <hyperlink ref="H639" r:id="rId538"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13875,7 +17443,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="D1:L132"/>
+  <dimension ref="D1:L165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -16027,8 +19595,470 @@
         <v>30.719612903225801</v>
       </c>
     </row>
+    <row r="136" spans="4:12">
+      <c r="D136" s="27">
+        <v>46235</v>
+      </c>
+      <c r="E136" s="28"/>
+      <c r="F136" s="28"/>
+      <c r="G136" s="28"/>
+      <c r="H136" s="28"/>
+      <c r="I136" s="28"/>
+      <c r="J136" s="28"/>
+      <c r="K136" s="28"/>
+      <c r="L136" s="28"/>
+    </row>
+    <row r="137" spans="4:12">
+      <c r="D137" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G137" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I137" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J137" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K137" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L137" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="4:12">
+      <c r="D138" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E138" s="10">
+        <v>46265</v>
+      </c>
+      <c r="F138" s="8">
+        <v>112</v>
+      </c>
+      <c r="G138" s="4">
+        <v>40.497301136363603</v>
+      </c>
+      <c r="I138" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="J138" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K138" s="8">
+        <v>96</v>
+      </c>
+      <c r="L138" s="4">
+        <v>37.910187317890497</v>
+      </c>
+    </row>
+    <row r="139" spans="4:12">
+      <c r="I139" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="J139" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K139" s="8">
+        <v>56</v>
+      </c>
+      <c r="L139" s="4">
+        <v>37.2749375</v>
+      </c>
+    </row>
+    <row r="140" spans="4:12">
+      <c r="I140" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="J140" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K140" s="8">
+        <v>136</v>
+      </c>
+      <c r="L140" s="4">
+        <v>31.938663606654799</v>
+      </c>
+    </row>
+    <row r="141" spans="4:12">
+      <c r="I141" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="J141" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K141" s="8">
+        <v>88</v>
+      </c>
+      <c r="L141" s="4">
+        <v>31.922168861024002</v>
+      </c>
+    </row>
+    <row r="142" spans="4:12">
+      <c r="I142" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="J142" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K142" s="8">
+        <v>136</v>
+      </c>
+      <c r="L142" s="4">
+        <v>31.604892504530302</v>
+      </c>
+    </row>
+    <row r="143" spans="4:12">
+      <c r="I143" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="J143" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K143" s="8">
+        <v>136</v>
+      </c>
+      <c r="L143" s="4">
+        <v>31.394258064516102</v>
+      </c>
+    </row>
+    <row r="144" spans="4:12">
+      <c r="I144" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="J144" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K144" s="8">
+        <v>160</v>
+      </c>
+      <c r="L144" s="4">
+        <v>29.823340469051601</v>
+      </c>
+    </row>
+    <row r="145" spans="4:12">
+      <c r="I145" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="J145" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K145" s="8">
+        <v>64</v>
+      </c>
+      <c r="L145" s="4">
+        <v>29.055033333333299</v>
+      </c>
+    </row>
+    <row r="146" spans="4:12">
+      <c r="I146" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="J146" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K146" s="8">
+        <v>136</v>
+      </c>
+      <c r="L146" s="4">
+        <v>28.483891129032301</v>
+      </c>
+    </row>
+    <row r="147" spans="4:12">
+      <c r="I147" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="J147" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K147" s="8">
+        <v>144</v>
+      </c>
+      <c r="L147" s="4">
+        <v>28.453307923980599</v>
+      </c>
+    </row>
+    <row r="148" spans="4:12">
+      <c r="I148" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J148" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K148" s="8">
+        <v>88</v>
+      </c>
+      <c r="L148" s="4">
+        <v>26.892847222222201</v>
+      </c>
+    </row>
+    <row r="149" spans="4:12">
+      <c r="I149" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J149" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K149" s="8">
+        <v>168</v>
+      </c>
+      <c r="L149" s="4">
+        <v>24.878616379310301</v>
+      </c>
+    </row>
+    <row r="150" spans="4:12">
+      <c r="I150" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="J150" s="10">
+        <v>46265</v>
+      </c>
+      <c r="K150" s="26">
+        <v>72</v>
+      </c>
+      <c r="L150" s="4">
+        <v>23.965367647058802</v>
+      </c>
+    </row>
+    <row r="154" spans="4:12">
+      <c r="D154" s="27">
+        <v>46266</v>
+      </c>
+      <c r="E154" s="28"/>
+      <c r="F154" s="28"/>
+      <c r="G154" s="28"/>
+      <c r="H154" s="28"/>
+      <c r="I154" s="28"/>
+      <c r="J154" s="28"/>
+      <c r="K154" s="28"/>
+      <c r="L154" s="28"/>
+    </row>
+    <row r="155" spans="4:12">
+      <c r="D155" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G155" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I155" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J155" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="K155" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="L155" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="4:12">
+      <c r="D156" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E156" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F156" s="8">
+        <v>112</v>
+      </c>
+      <c r="G156" s="4">
+        <v>49.117546875000002</v>
+      </c>
+      <c r="I156" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="J156" s="10">
+        <v>46295</v>
+      </c>
+      <c r="K156" s="8">
+        <v>192</v>
+      </c>
+      <c r="L156" s="4">
+        <v>36.709279166666697</v>
+      </c>
+    </row>
+    <row r="157" spans="4:12">
+      <c r="D157" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E157" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F157" s="8">
+        <v>168</v>
+      </c>
+      <c r="G157" s="4">
+        <v>45.8907234848485</v>
+      </c>
+      <c r="I157" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="J157" s="10">
+        <v>46295</v>
+      </c>
+      <c r="K157" s="8">
+        <v>168</v>
+      </c>
+      <c r="L157" s="4">
+        <v>36.1385890314547</v>
+      </c>
+    </row>
+    <row r="158" spans="4:12">
+      <c r="D158" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E158" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F158" s="8">
+        <v>120</v>
+      </c>
+      <c r="G158" s="4">
+        <v>45.193713573232301</v>
+      </c>
+      <c r="I158" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="J158" s="10">
+        <v>46295</v>
+      </c>
+      <c r="K158" s="8">
+        <v>200</v>
+      </c>
+      <c r="L158" s="4">
+        <v>33.869991249999998</v>
+      </c>
+    </row>
+    <row r="159" spans="4:12">
+      <c r="D159" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E159" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F159" s="8">
+        <v>168</v>
+      </c>
+      <c r="G159" s="4">
+        <v>42.752038640873003</v>
+      </c>
+      <c r="I159" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="J159" s="10">
+        <v>46295</v>
+      </c>
+      <c r="K159" s="26">
+        <v>152</v>
+      </c>
+      <c r="L159" s="4">
+        <v>33.735907565789503</v>
+      </c>
+    </row>
+    <row r="160" spans="4:12">
+      <c r="D160" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E160" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F160" s="8">
+        <v>176</v>
+      </c>
+      <c r="G160" s="4">
+        <v>42.457833333333298</v>
+      </c>
+    </row>
+    <row r="161" spans="4:7">
+      <c r="D161" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E161" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F161" s="8">
+        <v>184</v>
+      </c>
+      <c r="G161" s="4">
+        <v>41.455352356177102</v>
+      </c>
+    </row>
+    <row r="162" spans="4:7">
+      <c r="D162" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E162" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F162" s="8">
+        <v>176</v>
+      </c>
+      <c r="G162" s="4">
+        <v>40.9208262195122</v>
+      </c>
+    </row>
+    <row r="163" spans="4:7">
+      <c r="D163" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E163" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F163" s="8">
+        <v>104</v>
+      </c>
+      <c r="G163" s="4">
+        <v>40.9208262195122</v>
+      </c>
+    </row>
+    <row r="164" spans="4:7">
+      <c r="D164" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E164" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F164" s="8">
+        <v>184</v>
+      </c>
+      <c r="G164" s="4">
+        <v>40.175800000000002</v>
+      </c>
+    </row>
+    <row r="165" spans="4:7">
+      <c r="D165" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="E165" s="10">
+        <v>46295</v>
+      </c>
+      <c r="F165" s="8">
+        <v>152</v>
+      </c>
+      <c r="G165" s="4">
+        <v>39.802379807692297</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="D136:L136"/>
+    <mergeCell ref="D154:L154"/>
     <mergeCell ref="D122:L122"/>
     <mergeCell ref="D109:L109"/>
     <mergeCell ref="D50:L50"/>
@@ -16043,7 +20073,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -16276,10 +20306,430 @@
         <v>30.719612903225801</v>
       </c>
     </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C20" s="8">
+        <v>112</v>
+      </c>
+      <c r="D20" s="4">
+        <v>40.497301136363603</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C21" s="8">
+        <v>96</v>
+      </c>
+      <c r="D21" s="4">
+        <v>37.910187317890497</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C22" s="8">
+        <v>56</v>
+      </c>
+      <c r="D22" s="4">
+        <v>37.2749375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C23" s="8">
+        <v>136</v>
+      </c>
+      <c r="D23" s="4">
+        <v>31.938663606654799</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C24" s="8">
+        <v>88</v>
+      </c>
+      <c r="D24" s="4">
+        <v>31.922168861024002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C25" s="8">
+        <v>136</v>
+      </c>
+      <c r="D25" s="4">
+        <v>31.604892504530302</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C26" s="8">
+        <v>136</v>
+      </c>
+      <c r="D26" s="4">
+        <v>31.394258064516102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C27" s="8">
+        <v>160</v>
+      </c>
+      <c r="D27" s="4">
+        <v>29.823340469051601</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C28" s="8">
+        <v>64</v>
+      </c>
+      <c r="D28" s="4">
+        <v>29.055033333333299</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C29" s="8">
+        <v>136</v>
+      </c>
+      <c r="D29" s="4">
+        <v>28.483891129032301</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C30" s="8">
+        <v>144</v>
+      </c>
+      <c r="D30" s="4">
+        <v>28.453307923980599</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C31" s="8">
+        <v>88</v>
+      </c>
+      <c r="D31" s="4">
+        <v>26.892847222222201</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C32" s="8">
+        <v>168</v>
+      </c>
+      <c r="D32" s="4">
+        <v>24.878616379310301</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C33" s="26">
+        <v>72</v>
+      </c>
+      <c r="D33" s="4">
+        <v>23.965367647058802</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B37" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C37" s="8">
+        <v>112</v>
+      </c>
+      <c r="D37" s="4">
+        <v>49.117546875000002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C38" s="8">
+        <v>168</v>
+      </c>
+      <c r="D38" s="4">
+        <v>45.8907234848485</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C39" s="8">
+        <v>120</v>
+      </c>
+      <c r="D39" s="4">
+        <v>45.193713573232301</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C40" s="8">
+        <v>168</v>
+      </c>
+      <c r="D40" s="4">
+        <v>42.752038640873003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B41" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C41" s="8">
+        <v>176</v>
+      </c>
+      <c r="D41" s="4">
+        <v>42.457833333333298</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C42" s="8">
+        <v>184</v>
+      </c>
+      <c r="D42" s="4">
+        <v>41.455352356177102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C43" s="8">
+        <v>176</v>
+      </c>
+      <c r="D43" s="4">
+        <v>40.9208262195122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C44" s="8">
+        <v>104</v>
+      </c>
+      <c r="D44" s="4">
+        <v>40.9208262195122</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C45" s="8">
+        <v>184</v>
+      </c>
+      <c r="D45" s="4">
+        <v>40.175800000000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B46" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C46" s="8">
+        <v>152</v>
+      </c>
+      <c r="D46" s="4">
+        <v>39.802379807692297</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B47" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C47" s="8">
+        <v>192</v>
+      </c>
+      <c r="D47" s="4">
+        <v>36.709279166666697</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B48" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C48" s="8">
+        <v>168</v>
+      </c>
+      <c r="D48" s="4">
+        <v>36.1385890314547</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C49" s="8">
+        <v>200</v>
+      </c>
+      <c r="D49" s="4">
+        <v>33.869991249999998</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="B50" s="10">
+        <v>46295</v>
+      </c>
+      <c r="C50" s="26">
+        <v>152</v>
+      </c>
+      <c r="D50" s="4">
+        <v>33.735907565789503</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D16">
-    <sortState ref="A2:D16">
-      <sortCondition descending="1" ref="D1:D16"/>
+  <autoFilter ref="A36:D36">
+    <sortState ref="A37:D50">
+      <sortCondition descending="1" ref="D36"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>